<commit_message>
Atualiza artefactos da jornada sem descricao de cartoes
</commit_message>
<xml_diff>
--- a/public/templates/girabola_modelo_rodada_exemplo.xlsx
+++ b/public/templates/girabola_modelo_rodada_exemplo.xlsx
@@ -4274,7 +4274,9 @@
       <c r="K8" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="L8" s="7" t="n"/>
+      <c r="L8" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="M8" s="7" t="n"/>
       <c r="N8" s="7" t="n"/>
       <c r="O8" s="7" t="n"/>
@@ -4309,7 +4311,9 @@
       <c r="K9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="7" t="n"/>
+      <c r="L9" s="7" t="n">
+        <v>0</v>
+      </c>
       <c r="M9" s="7" t="n"/>
       <c r="N9" s="7" t="n"/>
       <c r="O9" s="7" t="n"/>

</xml_diff>